<commit_message>
Write Forecast Pro forecast into the shared Excel, add per-group SKU view and Render service.
</commit_message>
<xml_diff>
--- a/data/sources/inventarios.xlsx
+++ b/data/sources/inventarios.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/097b992f5ca9b29c/Desktop/OneDrive/Documents/LRI SupplyChain optimization/data/sources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/097b992f5ca9b29c/Documents/LRI SupplyChain optimization/data/sources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="72" documentId="11_5C0955DB1657F95119C1D6F0505ED87656CE6A58" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0D7A26A7-7550-4823-9358-ED4424D66665}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="11_5C0955DB1657F95119C1D6F0505ED87656CE6A58" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE772E62-269F-4E10-8FCD-CBAB48ED38C2}"/>
   <bookViews>
     <workbookView xWindow="-104" yWindow="-104" windowWidth="22326" windowHeight="13306" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="303">
   <si>
     <t>codigo</t>
   </si>
@@ -940,12 +940,18 @@
   </si>
   <si>
     <t>pronostico ajustado</t>
+  </si>
+  <si>
+    <t>A+</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1006,7 +1012,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -1016,6 +1022,7 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1032,10 +1039,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1323,7 +1326,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AV106"/>
+  <dimension ref="A1:AW106"/>
   <sheetFormatPr defaultColWidth="13.796875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="23" max="23" width="13.09765625" customWidth="1"/>
@@ -1332,7 +1335,7 @@
     <col min="30" max="30" width="16.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1477,8 +1480,13 @@
       <c r="AV1" t="s">
         <v>43</v>
       </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>fill rate deseado</t>
+        </is>
+      </c>
     </row>
-    <row r="2" spans="1:48" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>34041032</v>
       </c>
@@ -1486,7 +1494,7 @@
         <v>44</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>302</v>
       </c>
       <c r="D2" t="s">
         <v>46</v>
@@ -1546,8 +1554,7 @@
         <v>168.41508492361751</v>
       </c>
       <c r="W2" s="6">
-        <f>AVERAGE(K2:V2)</f>
-        <v>151.61252273755963</v>
+        <v>232.11964947684825</v>
       </c>
       <c r="X2" s="6">
         <f>_xlfn.STDEV.S(K2:V2)</f>
@@ -1557,8 +1564,8 @@
         <v>0.8</v>
       </c>
       <c r="Z2" s="6">
-        <f>NORMINV(Y2,W2,X2)</f>
-        <v>176.27114648275182</v>
+        <f>W2</f>
+        <v>232.11964947684825</v>
       </c>
       <c r="AA2" s="6">
         <v>21.51402325510422</v>
@@ -1623,8 +1630,11 @@
       <c r="AU2">
         <v>1.5</v>
       </c>
+      <c r="AW2" s="7">
+        <v>0.997</v>
+      </c>
     </row>
-    <row r="3" spans="1:48" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>50</v>
       </c>
@@ -1632,7 +1642,7 @@
         <v>44</v>
       </c>
       <c r="C3" t="s">
-        <v>45</v>
+        <v>302</v>
       </c>
       <c r="D3" t="s">
         <v>46</v>
@@ -1692,19 +1702,18 @@
         <v>147.7200786815956</v>
       </c>
       <c r="W3" s="6">
-        <f t="shared" ref="W3:W66" si="0">AVERAGE(K3:V3)</f>
-        <v>145.4553686620784</v>
+        <v>239.9456058938427</v>
       </c>
       <c r="X3" s="6">
-        <f t="shared" ref="X3:X66" si="1">_xlfn.STDEV.S(K3:V3)</f>
+        <f t="shared" ref="X3:X4" si="1">_xlfn.STDEV.S(K3:V3)</f>
         <v>34.387829298313072</v>
       </c>
       <c r="Y3" s="5">
         <v>0.8</v>
       </c>
       <c r="Z3" s="6">
-        <f>NORMINV(Y3,W3,X3)</f>
-        <v>174.39689597601947</v>
+        <f>W3</f>
+        <v>239.9456058938427</v>
       </c>
       <c r="AA3" s="6">
         <v>83.437299722281566</v>
@@ -1769,8 +1778,11 @@
       <c r="AU3">
         <v>1.5</v>
       </c>
+      <c r="AW3" s="7">
+        <v>0.997</v>
+      </c>
     </row>
-    <row r="4" spans="1:48" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>77001046</v>
       </c>
@@ -1778,7 +1790,7 @@
         <v>52</v>
       </c>
       <c r="C4" t="s">
-        <v>45</v>
+        <v>302</v>
       </c>
       <c r="D4" t="s">
         <v>53</v>
@@ -1838,8 +1850,7 @@
         <v>128.36066540912731</v>
       </c>
       <c r="W4" s="6">
-        <f t="shared" si="0"/>
-        <v>157.90283820606416</v>
+        <v>280.39424132948034</v>
       </c>
       <c r="X4" s="6">
         <f t="shared" si="1"/>
@@ -1849,8 +1860,8 @@
         <v>0.8</v>
       </c>
       <c r="Z4" s="6">
-        <f t="shared" ref="Z4:Z67" si="2">NORMINV(Y4,W4,X4)</f>
-        <v>195.42087597460073</v>
+        <f>W4</f>
+        <v>280.39424132948034</v>
       </c>
       <c r="AA4" s="6">
         <v>65.184789574877158</v>
@@ -1915,8 +1926,11 @@
       <c r="AU4">
         <v>1.5</v>
       </c>
+      <c r="AW4" s="7">
+        <v>0.997</v>
+      </c>
     </row>
-    <row r="5" spans="1:48" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>55</v>
       </c>
@@ -1924,7 +1938,7 @@
         <v>56</v>
       </c>
       <c r="C5" t="s">
-        <v>45</v>
+        <v>302</v>
       </c>
       <c r="D5" t="s">
         <v>57</v>
@@ -1984,8 +1998,7 @@
         <v>171.38415311492281</v>
       </c>
       <c r="W5" s="6">
-        <f t="shared" ref="W5:W68" si="3">AVERAGE(K5:V5)</f>
-        <v>153.17944568450912</v>
+        <v>229.22550358106025</v>
       </c>
       <c r="X5" s="6">
         <f t="shared" ref="X5:X68" si="4">_xlfn.STDEV.S(K5:V5)</f>
@@ -1995,8 +2008,8 @@
         <v>0.8</v>
       </c>
       <c r="Z5" s="6">
-        <f t="shared" si="2"/>
-        <v>176.47168334004874</v>
+        <f>W5</f>
+        <v>229.22550358106025</v>
       </c>
       <c r="AA5" s="6">
         <v>85.734733115634626</v>
@@ -2061,8 +2074,11 @@
       <c r="AU5">
         <v>1.5</v>
       </c>
+      <c r="AW5" s="7">
+        <v>0.997</v>
+      </c>
     </row>
-    <row r="6" spans="1:48" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>59</v>
       </c>
@@ -2070,7 +2086,7 @@
         <v>52</v>
       </c>
       <c r="C6" t="s">
-        <v>45</v>
+        <v>302</v>
       </c>
       <c r="D6" t="s">
         <v>53</v>
@@ -2130,8 +2146,7 @@
         <v>138.1544908930664</v>
       </c>
       <c r="W6" s="6">
-        <f t="shared" si="3"/>
-        <v>149.20629818461748</v>
+        <v>224.2772985482991</v>
       </c>
       <c r="X6" s="6">
         <f t="shared" si="4"/>
@@ -2141,8 +2156,8 @@
         <v>0.8</v>
       </c>
       <c r="Z6" s="6">
-        <f t="shared" si="2"/>
-        <v>172.19988430697288</v>
+        <f>W6</f>
+        <v>224.2772985482991</v>
       </c>
       <c r="AA6" s="6">
         <v>23.45744193853572</v>
@@ -2207,8 +2222,11 @@
       <c r="AU6">
         <v>1.5</v>
       </c>
+      <c r="AW6" s="7">
+        <v>0.997</v>
+      </c>
     </row>
-    <row r="7" spans="1:48" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>61</v>
       </c>
@@ -2216,7 +2234,7 @@
         <v>56</v>
       </c>
       <c r="C7" t="s">
-        <v>45</v>
+        <v>302</v>
       </c>
       <c r="D7" t="s">
         <v>57</v>
@@ -2276,8 +2294,7 @@
         <v>142.55874172376929</v>
       </c>
       <c r="W7" s="6">
-        <f t="shared" si="3"/>
-        <v>148.62260438021625</v>
+        <v>219.90973247373853</v>
       </c>
       <c r="X7" s="6">
         <f t="shared" si="4"/>
@@ -2287,8 +2304,8 @@
         <v>0.8</v>
       </c>
       <c r="Z7" s="6">
-        <f t="shared" si="2"/>
-        <v>170.45722375777788</v>
+        <f>W7</f>
+        <v>219.90973247373853</v>
       </c>
       <c r="AA7" s="6">
         <v>58.177739799188203</v>
@@ -2353,8 +2370,11 @@
       <c r="AU7">
         <v>1.5</v>
       </c>
+      <c r="AW7" s="7">
+        <v>0.997</v>
+      </c>
     </row>
-    <row r="8" spans="1:48" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>63</v>
       </c>
@@ -2362,7 +2382,7 @@
         <v>64</v>
       </c>
       <c r="C8" t="s">
-        <v>45</v>
+        <v>302</v>
       </c>
       <c r="D8" t="s">
         <v>65</v>
@@ -2422,8 +2442,7 @@
         <v>169.60456756933129</v>
       </c>
       <c r="W8" s="6">
-        <f t="shared" si="3"/>
-        <v>162.13731195548462</v>
+        <v>221.66185300665364</v>
       </c>
       <c r="X8" s="6">
         <f t="shared" si="4"/>
@@ -2433,8 +2452,8 @@
         <v>0.8</v>
       </c>
       <c r="Z8" s="6">
-        <f t="shared" si="2"/>
-        <v>180.3691545368163</v>
+        <f>W8</f>
+        <v>221.66185300665364</v>
       </c>
       <c r="AA8" s="6">
         <v>10.0122074037904</v>
@@ -2499,8 +2518,11 @@
       <c r="AU8">
         <v>1.5</v>
       </c>
+      <c r="AW8" s="7">
+        <v>0.997</v>
+      </c>
     </row>
-    <row r="9" spans="1:48" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>67</v>
       </c>
@@ -2508,7 +2530,7 @@
         <v>52</v>
       </c>
       <c r="C9" t="s">
-        <v>45</v>
+        <v>302</v>
       </c>
       <c r="D9" t="s">
         <v>53</v>
@@ -2568,8 +2590,7 @@
         <v>118.9969854443916</v>
       </c>
       <c r="W9" s="6">
-        <f t="shared" si="3"/>
-        <v>169.11924698561052</v>
+        <v>256.9347343529299</v>
       </c>
       <c r="X9" s="6">
         <f t="shared" si="4"/>
@@ -2579,8 +2600,8 @@
         <v>0.8</v>
       </c>
       <c r="Z9" s="6">
-        <f t="shared" si="2"/>
-        <v>196.01635721292973</v>
+        <f>W9</f>
+        <v>256.9347343529299</v>
       </c>
       <c r="AA9" s="6">
         <v>10.32227546006653</v>
@@ -2645,8 +2666,11 @@
       <c r="AU9">
         <v>1.5</v>
       </c>
+      <c r="AW9" s="7">
+        <v>0.997</v>
+      </c>
     </row>
-    <row r="10" spans="1:48" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>69</v>
       </c>
@@ -2654,7 +2678,7 @@
         <v>64</v>
       </c>
       <c r="C10" t="s">
-        <v>45</v>
+        <v>302</v>
       </c>
       <c r="D10" t="s">
         <v>70</v>
@@ -2714,8 +2738,7 @@
         <v>113.90795331535629</v>
       </c>
       <c r="W10" s="6">
-        <f t="shared" si="3"/>
-        <v>136.66705209870997</v>
+        <v>227.33445488586847</v>
       </c>
       <c r="X10" s="6">
         <f t="shared" si="4"/>
@@ -2725,8 +2748,8 @@
         <v>0.8</v>
       </c>
       <c r="Z10" s="6">
-        <f t="shared" si="2"/>
-        <v>164.43767889703619</v>
+        <f>W10</f>
+        <v>227.33445488586847</v>
       </c>
       <c r="AA10" s="6">
         <v>11.157261879329811</v>
@@ -2791,8 +2814,11 @@
       <c r="AU10">
         <v>1.5</v>
       </c>
+      <c r="AW10" s="7">
+        <v>0.997</v>
+      </c>
     </row>
-    <row r="11" spans="1:48" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>73</v>
       </c>
@@ -2800,7 +2826,7 @@
         <v>44</v>
       </c>
       <c r="C11" t="s">
-        <v>45</v>
+        <v>302</v>
       </c>
       <c r="D11" t="s">
         <v>46</v>
@@ -2860,8 +2886,7 @@
         <v>90.043198876082897</v>
       </c>
       <c r="W11" s="6">
-        <f t="shared" si="3"/>
-        <v>145.82410339371563</v>
+        <v>236.077038822022</v>
       </c>
       <c r="X11" s="6">
         <f t="shared" si="4"/>
@@ -2871,8 +2896,8 @@
         <v>0.8</v>
       </c>
       <c r="Z11" s="6">
-        <f t="shared" si="2"/>
-        <v>173.46778249100547</v>
+        <f>W11</f>
+        <v>236.077038822022</v>
       </c>
       <c r="AA11" s="6">
         <v>22.903225806451609</v>
@@ -2937,8 +2962,11 @@
       <c r="AU11">
         <v>1.5</v>
       </c>
+      <c r="AW11" s="7">
+        <v>0.997</v>
+      </c>
     </row>
-    <row r="12" spans="1:48" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>75</v>
       </c>
@@ -2946,7 +2974,7 @@
         <v>64</v>
       </c>
       <c r="C12" t="s">
-        <v>45</v>
+        <v>302</v>
       </c>
       <c r="D12" t="s">
         <v>65</v>
@@ -3006,8 +3034,7 @@
         <v>178.50358669093109</v>
       </c>
       <c r="W12" s="6">
-        <f t="shared" si="3"/>
-        <v>164.71245525408449</v>
+        <v>238.9726240353031</v>
       </c>
       <c r="X12" s="6">
         <f t="shared" si="4"/>
@@ -3017,8 +3044,8 @@
         <v>0.8</v>
       </c>
       <c r="Z12" s="6">
-        <f t="shared" si="2"/>
-        <v>187.45769080522379</v>
+        <f>W12</f>
+        <v>238.9726240353031</v>
       </c>
       <c r="AA12" s="6">
         <v>53.424176763206887</v>
@@ -3083,8 +3110,11 @@
       <c r="AU12">
         <v>1.5</v>
       </c>
+      <c r="AW12" s="7">
+        <v>0.997</v>
+      </c>
     </row>
-    <row r="13" spans="1:48" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>78</v>
       </c>
@@ -3092,7 +3122,7 @@
         <v>44</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>302</v>
       </c>
       <c r="D13" t="s">
         <v>79</v>
@@ -3152,8 +3182,7 @@
         <v>162.99317773373329</v>
       </c>
       <c r="W13" s="6">
-        <f t="shared" si="3"/>
-        <v>163.81432639391278</v>
+        <v>263.27348420163725</v>
       </c>
       <c r="X13" s="6">
         <f t="shared" si="4"/>
@@ -3163,8 +3192,8 @@
         <v>0.8</v>
       </c>
       <c r="Z13" s="6">
-        <f t="shared" si="2"/>
-        <v>194.27779030980375</v>
+        <f>W13</f>
+        <v>263.27348420163725</v>
       </c>
       <c r="AA13" s="6">
         <v>21.03793450727866</v>
@@ -3229,8 +3258,11 @@
       <c r="AU13">
         <v>1.5</v>
       </c>
+      <c r="AW13" s="7">
+        <v>0.997</v>
+      </c>
     </row>
-    <row r="14" spans="1:48" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>81</v>
       </c>
@@ -3238,7 +3270,7 @@
         <v>56</v>
       </c>
       <c r="C14" t="s">
-        <v>45</v>
+        <v>302</v>
       </c>
       <c r="D14" t="s">
         <v>57</v>
@@ -3298,8 +3330,7 @@
         <v>140.43932348286029</v>
       </c>
       <c r="W14" s="6">
-        <f t="shared" si="3"/>
-        <v>159.07278092654451</v>
+        <v>216.5821048351028</v>
       </c>
       <c r="X14" s="6">
         <f t="shared" si="4"/>
@@ -3309,8 +3340,8 @@
         <v>0.8</v>
       </c>
       <c r="Z14" s="6">
-        <f t="shared" si="2"/>
-        <v>176.68738024883629</v>
+        <f>W14</f>
+        <v>216.5821048351028</v>
       </c>
       <c r="AA14" s="6">
         <v>39.46378978850673</v>
@@ -3375,8 +3406,11 @@
       <c r="AU14">
         <v>1.5</v>
       </c>
+      <c r="AW14" s="7">
+        <v>0.997</v>
+      </c>
     </row>
-    <row r="15" spans="1:48" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>83</v>
       </c>
@@ -3384,7 +3418,7 @@
         <v>56</v>
       </c>
       <c r="C15" t="s">
-        <v>45</v>
+        <v>302</v>
       </c>
       <c r="D15" t="s">
         <v>57</v>
@@ -3444,8 +3478,7 @@
         <v>133.04577957242151</v>
       </c>
       <c r="W15" s="6">
-        <f t="shared" si="3"/>
-        <v>157.64358105698193</v>
+        <v>215.0504531040531</v>
       </c>
       <c r="X15" s="6">
         <f t="shared" si="4"/>
@@ -3455,8 +3488,8 @@
         <v>0.8</v>
       </c>
       <c r="Z15" s="6">
-        <f t="shared" si="2"/>
-        <v>175.22680027658294</v>
+        <f>W15</f>
+        <v>215.0504531040531</v>
       </c>
       <c r="AA15" s="6">
         <v>75.485396893215736</v>
@@ -3521,8 +3554,11 @@
       <c r="AU15">
         <v>1.5</v>
       </c>
+      <c r="AW15" s="7">
+        <v>0.997</v>
+      </c>
     </row>
-    <row r="16" spans="1:48" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>85</v>
       </c>
@@ -3530,7 +3566,7 @@
         <v>52</v>
       </c>
       <c r="C16" t="s">
-        <v>45</v>
+        <v>302</v>
       </c>
       <c r="D16" t="s">
         <v>86</v>
@@ -3590,8 +3626,7 @@
         <v>170.20804004132509</v>
       </c>
       <c r="W16" s="6">
-        <f t="shared" si="3"/>
-        <v>156.73083775382111</v>
+        <v>234.68536409270772</v>
       </c>
       <c r="X16" s="6">
         <f t="shared" si="4"/>
@@ -3601,8 +3636,8 @@
         <v>0.8</v>
       </c>
       <c r="Z16" s="6">
-        <f t="shared" si="2"/>
-        <v>180.60762248183948</v>
+        <f>W16</f>
+        <v>234.68536409270772</v>
       </c>
       <c r="AA16" s="6">
         <v>71.010162663655507</v>
@@ -3667,8 +3702,11 @@
       <c r="AU16">
         <v>1.5</v>
       </c>
+      <c r="AW16" s="7">
+        <v>0.997</v>
+      </c>
     </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>88</v>
       </c>
@@ -3676,7 +3714,7 @@
         <v>64</v>
       </c>
       <c r="C17" t="s">
-        <v>45</v>
+        <v>302</v>
       </c>
       <c r="D17" t="s">
         <v>65</v>
@@ -3736,8 +3774,7 @@
         <v>120.8114273744286</v>
       </c>
       <c r="W17" s="6">
-        <f t="shared" si="3"/>
-        <v>155.39505435881438</v>
+        <v>205.76086207928248</v>
       </c>
       <c r="X17" s="6">
         <f t="shared" si="4"/>
@@ -3747,8 +3784,8 @@
         <v>0.8</v>
       </c>
       <c r="Z17" s="6">
-        <f t="shared" si="2"/>
-        <v>170.82165759884325</v>
+        <f>W17</f>
+        <v>205.76086207928248</v>
       </c>
       <c r="AA17" s="6">
         <v>44.422437208166762</v>
@@ -3813,8 +3850,11 @@
       <c r="AU17">
         <v>1.5</v>
       </c>
+      <c r="AW17" s="7">
+        <v>0.997</v>
+      </c>
     </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>90</v>
       </c>
@@ -3882,8 +3922,7 @@
         <v>136.82002342320629</v>
       </c>
       <c r="W18" s="6">
-        <f t="shared" si="3"/>
-        <v>155.36137179096843</v>
+        <v>198.25781430853</v>
       </c>
       <c r="X18" s="6">
         <f t="shared" si="4"/>
@@ -3893,8 +3932,8 @@
         <v>0.8</v>
       </c>
       <c r="Z18" s="6">
-        <f t="shared" si="2"/>
-        <v>174.55675650040874</v>
+        <f>W18</f>
+        <v>198.25781430853</v>
       </c>
       <c r="AA18" s="6">
         <v>15.91326639606921</v>
@@ -3959,8 +3998,11 @@
       <c r="AU18">
         <v>1.5</v>
       </c>
+      <c r="AW18" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>92</v>
       </c>
@@ -4028,8 +4070,7 @@
         <v>162.06665274366969</v>
       </c>
       <c r="W19" s="6">
-        <f t="shared" si="3"/>
-        <v>155.21739877967775</v>
+        <v>207.79579762452053</v>
       </c>
       <c r="X19" s="6">
         <f t="shared" si="4"/>
@@ -4039,8 +4080,8 @@
         <v>0.8</v>
       </c>
       <c r="Z19" s="6">
-        <f t="shared" si="2"/>
-        <v>178.74528440375886</v>
+        <f>W19</f>
+        <v>207.79579762452053</v>
       </c>
       <c r="AA19" s="6">
         <v>11.845759453108309</v>
@@ -4105,8 +4146,11 @@
       <c r="AU19">
         <v>1.5</v>
       </c>
+      <c r="AW19" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>95</v>
       </c>
@@ -4174,8 +4218,7 @@
         <v>141.1346094449982</v>
       </c>
       <c r="W20" s="6">
-        <f t="shared" si="3"/>
-        <v>153.19798516557057</v>
+        <v>189.89089621352352</v>
       </c>
       <c r="X20" s="6">
         <f t="shared" si="4"/>
@@ -4185,8 +4228,8 @@
         <v>0.8</v>
       </c>
       <c r="Z20" s="6">
-        <f t="shared" si="2"/>
-        <v>169.61740137674911</v>
+        <f>W20</f>
+        <v>189.89089621352352</v>
       </c>
       <c r="AA20" s="6">
         <v>12.89315469832453</v>
@@ -4251,8 +4294,11 @@
       <c r="AU20">
         <v>1.5</v>
       </c>
+      <c r="AW20" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="21" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>97</v>
       </c>
@@ -4320,8 +4366,7 @@
         <v>142.68172814481659</v>
       </c>
       <c r="W21" s="6">
-        <f t="shared" si="3"/>
-        <v>153.10385814827896</v>
+        <v>221.41233412821532</v>
       </c>
       <c r="X21" s="6">
         <f t="shared" si="4"/>
@@ -4331,8 +4376,8 @@
         <v>0.8</v>
       </c>
       <c r="Z21" s="6">
-        <f t="shared" si="2"/>
-        <v>183.67066971578015</v>
+        <f>W21</f>
+        <v>221.41233412821532</v>
       </c>
       <c r="AA21" s="6">
         <v>27.341837824640649</v>
@@ -4397,8 +4442,11 @@
       <c r="AU21">
         <v>1.5</v>
       </c>
+      <c r="AW21" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="22" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>99</v>
       </c>
@@ -4466,8 +4514,7 @@
         <v>132.2591234988067</v>
       </c>
       <c r="W22" s="6">
-        <f t="shared" si="3"/>
-        <v>151.64516222866951</v>
+        <v>205.8931173856467</v>
       </c>
       <c r="X22" s="6">
         <f t="shared" si="4"/>
@@ -4477,8 +4524,8 @@
         <v>0.8</v>
       </c>
       <c r="Z22" s="6">
-        <f t="shared" si="2"/>
-        <v>175.92014420444394</v>
+        <f>W22</f>
+        <v>205.8931173856467</v>
       </c>
       <c r="AA22" s="6">
         <v>65.572985015411845</v>
@@ -4543,8 +4590,11 @@
       <c r="AU22">
         <v>1.5</v>
       </c>
+      <c r="AW22" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="23" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>101</v>
       </c>
@@ -4612,8 +4662,7 @@
         <v>144.3825628179184</v>
       </c>
       <c r="W23" s="6">
-        <f t="shared" si="3"/>
-        <v>142.47978337280074</v>
+        <v>196.16192787055388</v>
       </c>
       <c r="X23" s="6">
         <f t="shared" si="4"/>
@@ -4623,8 +4672,8 @@
         <v>0.8</v>
       </c>
       <c r="Z23" s="6">
-        <f t="shared" si="2"/>
-        <v>166.50157527874447</v>
+        <f>W23</f>
+        <v>196.16192787055388</v>
       </c>
       <c r="AA23" s="6">
         <v>23.45500045777764</v>
@@ -4689,8 +4738,11 @@
       <c r="AU23">
         <v>1.5</v>
       </c>
+      <c r="AW23" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="24" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>103</v>
       </c>
@@ -4758,8 +4810,7 @@
         <v>106.88162925944199</v>
       </c>
       <c r="W24" s="6">
-        <f t="shared" si="3"/>
-        <v>150.60350089370331</v>
+        <v>206.92577641081417</v>
       </c>
       <c r="X24" s="6">
         <f t="shared" si="4"/>
@@ -4769,8 +4820,8 @@
         <v>0.8</v>
       </c>
       <c r="Z24" s="6">
-        <f t="shared" si="2"/>
-        <v>175.80670383575222</v>
+        <f>W24</f>
+        <v>206.92577641081417</v>
       </c>
       <c r="AA24" s="6">
         <v>55.61418500320444</v>
@@ -4835,8 +4886,11 @@
       <c r="AU24">
         <v>1.5</v>
       </c>
+      <c r="AW24" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="25" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>105</v>
       </c>
@@ -4904,8 +4958,7 @@
         <v>141.89418531386761</v>
       </c>
       <c r="W25" s="6">
-        <f t="shared" si="3"/>
-        <v>149.98303223947005</v>
+        <v>195.26889923631177</v>
       </c>
       <c r="X25" s="6">
         <f t="shared" si="4"/>
@@ -4915,8 +4968,8 @@
         <v>0.8</v>
       </c>
       <c r="Z25" s="6">
-        <f t="shared" si="2"/>
-        <v>170.24764132795204</v>
+        <f>W25</f>
+        <v>195.26889923631177</v>
       </c>
       <c r="AA25" s="6">
         <v>32.547074800866717</v>
@@ -4981,8 +5034,11 @@
       <c r="AU25">
         <v>1.5</v>
       </c>
+      <c r="AW25" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="26" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>107</v>
       </c>
@@ -5050,8 +5106,7 @@
         <v>143.6051835902617</v>
       </c>
       <c r="W26" s="6">
-        <f t="shared" si="3"/>
-        <v>149.92049026786844</v>
+        <v>203.57283786619493</v>
       </c>
       <c r="X26" s="6">
         <f t="shared" si="4"/>
@@ -5061,8 +5116,8 @@
         <v>0.8</v>
       </c>
       <c r="Z26" s="6">
-        <f t="shared" si="2"/>
-        <v>173.92894859848346</v>
+        <f>W26</f>
+        <v>203.57283786619493</v>
       </c>
       <c r="AA26" s="6">
         <v>68.285470137638484</v>
@@ -5127,8 +5182,11 @@
       <c r="AU26">
         <v>1.5</v>
       </c>
+      <c r="AW26" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="27" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>109</v>
       </c>
@@ -5196,8 +5254,7 @@
         <v>151.89575075637549</v>
       </c>
       <c r="W27" s="6">
-        <f t="shared" si="3"/>
-        <v>149.19103572665335</v>
+        <v>199.50929197857783</v>
       </c>
       <c r="X27" s="6">
         <f t="shared" si="4"/>
@@ -5207,8 +5264,8 @@
         <v>0.8</v>
       </c>
       <c r="Z27" s="6">
-        <f t="shared" si="2"/>
-        <v>171.70754828520566</v>
+        <f>W27</f>
+        <v>199.50929197857783</v>
       </c>
       <c r="AA27" s="6">
         <v>38.516495254371783</v>
@@ -5273,8 +5330,11 @@
       <c r="AU27">
         <v>1.5</v>
       </c>
+      <c r="AW27" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="28" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>111</v>
       </c>
@@ -5342,8 +5402,7 @@
         <v>158.45386693981709</v>
       </c>
       <c r="W28" s="6">
-        <f t="shared" si="3"/>
-        <v>147.49429662188049</v>
+        <v>198.11598908121806</v>
       </c>
       <c r="X28" s="6">
         <f t="shared" si="4"/>
@@ -5353,8 +5412,8 @@
         <v>0.8</v>
       </c>
       <c r="Z28" s="6">
-        <f t="shared" si="2"/>
-        <v>170.14659141304296</v>
+        <f>W28</f>
+        <v>198.11598908121806</v>
       </c>
       <c r="AA28" s="6">
         <v>28.53572191534165</v>
@@ -5419,8 +5478,11 @@
       <c r="AU28">
         <v>1.5</v>
       </c>
+      <c r="AW28" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="29" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>113</v>
       </c>
@@ -5488,8 +5550,7 @@
         <v>169.2789912034641</v>
       </c>
       <c r="W29" s="6">
-        <f t="shared" si="3"/>
-        <v>147.66229734632361</v>
+        <v>222.76536908888343</v>
       </c>
       <c r="X29" s="6">
         <f t="shared" si="4"/>
@@ -5499,8 +5560,8 @@
         <v>0.8</v>
       </c>
       <c r="Z29" s="6">
-        <f t="shared" si="2"/>
-        <v>181.26956802777798</v>
+        <f>W29</f>
+        <v>222.76536908888343</v>
       </c>
       <c r="AA29" s="6">
         <v>29.592883083590198</v>
@@ -5565,8 +5626,11 @@
       <c r="AU29">
         <v>1.5</v>
       </c>
+      <c r="AW29" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="30" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>115</v>
       </c>
@@ -5634,8 +5698,7 @@
         <v>171.9201297113614</v>
       </c>
       <c r="W30" s="6">
-        <f t="shared" si="3"/>
-        <v>142.9065381820692</v>
+        <v>189.04856883772447</v>
       </c>
       <c r="X30" s="6">
         <f t="shared" si="4"/>
@@ -5645,8 +5708,8 @@
         <v>0.8</v>
       </c>
       <c r="Z30" s="6">
-        <f t="shared" si="2"/>
-        <v>163.55426507334909</v>
+        <f>W30</f>
+        <v>189.04856883772447</v>
       </c>
       <c r="AA30" s="6">
         <v>26.951200903347878</v>
@@ -5711,8 +5774,11 @@
       <c r="AU30">
         <v>1.5</v>
       </c>
+      <c r="AW30" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="31" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>118</v>
       </c>
@@ -5780,8 +5846,7 @@
         <v>127.4333900859347</v>
       </c>
       <c r="W31" s="6">
-        <f t="shared" si="3"/>
-        <v>141.86140655638155</v>
+        <v>193.28067867738974</v>
       </c>
       <c r="X31" s="6">
         <f t="shared" si="4"/>
@@ -5791,8 +5856,8 @@
         <v>0.8</v>
       </c>
       <c r="Z31" s="6">
-        <f t="shared" si="2"/>
-        <v>164.87060386774556</v>
+        <f>W31</f>
+        <v>193.28067867738974</v>
       </c>
       <c r="AA31" s="6">
         <v>19.38261055330058</v>
@@ -5857,8 +5922,11 @@
       <c r="AU31">
         <v>1.5</v>
       </c>
+      <c r="AW31" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="32" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>120</v>
       </c>
@@ -5926,8 +5994,7 @@
         <v>121.69040852895709</v>
       </c>
       <c r="W32" s="6">
-        <f t="shared" si="3"/>
-        <v>164.72866699714359</v>
+        <v>214.05725493961467</v>
       </c>
       <c r="X32" s="6">
         <f t="shared" si="4"/>
@@ -5937,8 +6004,8 @@
         <v>0.8</v>
       </c>
       <c r="Z32" s="6">
-        <f t="shared" si="2"/>
-        <v>186.80232082849682</v>
+        <f>W32</f>
+        <v>214.05725493961467</v>
       </c>
       <c r="AA32" s="6">
         <v>54.830469679860833</v>
@@ -6003,8 +6070,11 @@
       <c r="AU32">
         <v>1.5</v>
       </c>
+      <c r="AW32" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="33" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>122</v>
       </c>
@@ -6072,8 +6142,7 @@
         <v>136.7087353777606</v>
       </c>
       <c r="W33" s="6">
-        <f t="shared" si="3"/>
-        <v>138.31068808158307</v>
+        <v>207.47326592415635</v>
       </c>
       <c r="X33" s="6">
         <f t="shared" si="4"/>
@@ -6083,8 +6152,8 @@
         <v>0.8</v>
       </c>
       <c r="Z33" s="6">
-        <f t="shared" si="2"/>
-        <v>169.259694835262</v>
+        <f>W33</f>
+        <v>207.47326592415635</v>
       </c>
       <c r="AA33" s="6">
         <v>56.424756614886931</v>
@@ -6149,8 +6218,11 @@
       <c r="AU33">
         <v>1.5</v>
       </c>
+      <c r="AW33" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="34" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>125</v>
       </c>
@@ -6218,8 +6290,7 @@
         <v>181.3693817588501</v>
       </c>
       <c r="W34" s="6">
-        <f t="shared" si="3"/>
-        <v>150.58600164720701</v>
+        <v>206.9437055356384</v>
       </c>
       <c r="X34" s="6">
         <f t="shared" si="4"/>
@@ -6229,8 +6300,8 @@
         <v>0.8</v>
       </c>
       <c r="Z34" s="6">
-        <f t="shared" si="2"/>
-        <v>175.8050581467356</v>
+        <f>W34</f>
+        <v>206.9437055356384</v>
       </c>
       <c r="AA34" s="6">
         <v>16.508987701040681</v>
@@ -6295,8 +6366,11 @@
       <c r="AU34">
         <v>1.5</v>
       </c>
+      <c r="AW34" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="35" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>127</v>
       </c>
@@ -6364,8 +6438,7 @@
         <v>138.0824930187373</v>
       </c>
       <c r="W35" s="6">
-        <f t="shared" si="3"/>
-        <v>132.44301764316333</v>
+        <v>175.77304596083</v>
       </c>
       <c r="X35" s="6">
         <f t="shared" si="4"/>
@@ -6375,8 +6448,8 @@
         <v>0.8</v>
       </c>
       <c r="Z35" s="6">
-        <f t="shared" si="2"/>
-        <v>151.83242418166714</v>
+        <f>W35</f>
+        <v>175.77304596083</v>
       </c>
       <c r="AA35" s="6">
         <v>14.10168767357402</v>
@@ -6441,8 +6514,11 @@
       <c r="AU35">
         <v>1.5</v>
       </c>
+      <c r="AW35" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="36" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>129</v>
       </c>
@@ -6510,8 +6586,7 @@
         <v>97.944070299854502</v>
       </c>
       <c r="W36" s="6">
-        <f t="shared" si="3"/>
-        <v>131.77401892007765</v>
+        <v>197.47345518083807</v>
       </c>
       <c r="X36" s="6">
         <f t="shared" si="4"/>
@@ -6521,8 +6596,8 @@
         <v>0.8</v>
       </c>
       <c r="Z36" s="6">
-        <f t="shared" si="2"/>
-        <v>161.17333224780543</v>
+        <f>W36</f>
+        <v>197.47345518083807</v>
       </c>
       <c r="AA36" s="6">
         <v>65.314188055055382</v>
@@ -6587,8 +6662,11 @@
       <c r="AU36">
         <v>1.5</v>
       </c>
+      <c r="AW36" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="37" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>131</v>
       </c>
@@ -6656,8 +6734,7 @@
         <v>149.86343937052879</v>
       </c>
       <c r="W37" s="6">
-        <f t="shared" si="3"/>
-        <v>162.56504162938651</v>
+        <v>207.68108748641214</v>
       </c>
       <c r="X37" s="6">
         <f t="shared" si="4"/>
@@ -6667,8 +6744,8 @@
         <v>0.8</v>
       </c>
       <c r="Z37" s="6">
-        <f t="shared" si="2"/>
-        <v>182.75365881925779</v>
+        <f>W37</f>
+        <v>207.68108748641214</v>
       </c>
       <c r="AA37" s="6">
         <v>85.856807153538625</v>
@@ -6733,8 +6810,11 @@
       <c r="AU37">
         <v>1.5</v>
       </c>
+      <c r="AW37" s="7">
+        <v>0.97</v>
+      </c>
     </row>
-    <row r="38" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>28260020</v>
       </c>
@@ -6802,8 +6882,7 @@
         <v>168.2850726559991</v>
       </c>
       <c r="W38" s="6">
-        <f t="shared" si="3"/>
-        <v>153.99870430101146</v>
+        <v>179.03165202697022</v>
       </c>
       <c r="X38" s="6">
         <f t="shared" si="4"/>
@@ -6813,8 +6892,8 @@
         <v>0.8</v>
       </c>
       <c r="Z38" s="6">
-        <f t="shared" si="2"/>
-        <v>170.43835519881566</v>
+        <f>W38</f>
+        <v>179.03165202697022</v>
       </c>
       <c r="AA38" s="6">
         <v>25.28122806482131</v>
@@ -6879,8 +6958,11 @@
       <c r="AU38">
         <v>0.5</v>
       </c>
+      <c r="AW38" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="39" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>136</v>
       </c>
@@ -6948,8 +7030,7 @@
         <v>134.70057107624601</v>
       </c>
       <c r="W39" s="6">
-        <f t="shared" si="3"/>
-        <v>152.48484468556853</v>
+        <v>193.98651555502894</v>
       </c>
       <c r="X39" s="6">
         <f t="shared" si="4"/>
@@ -6959,8 +7040,8 @@
         <v>0.8</v>
       </c>
       <c r="Z39" s="6">
-        <f t="shared" si="2"/>
-        <v>179.73984430600856</v>
+        <f>W39</f>
+        <v>193.98651555502894</v>
       </c>
       <c r="AA39" s="6">
         <v>60.340891750846893</v>
@@ -7025,8 +7106,11 @@
       <c r="AU39">
         <v>0.5</v>
       </c>
+      <c r="AW39" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="40" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>138</v>
       </c>
@@ -7094,8 +7178,7 @@
         <v>165.2915845319512</v>
       </c>
       <c r="W40" s="6">
-        <f t="shared" si="3"/>
-        <v>146.03727189878555</v>
+        <v>179.71585223517022</v>
       </c>
       <c r="X40" s="6">
         <f t="shared" si="4"/>
@@ -7105,8 +7188,8 @@
         <v>0.8</v>
       </c>
       <c r="Z40" s="6">
-        <f t="shared" si="2"/>
-        <v>168.15468729568181</v>
+        <f>W40</f>
+        <v>179.71585223517022</v>
       </c>
       <c r="AA40" s="6">
         <v>81.288796655171353</v>
@@ -7171,8 +7254,11 @@
       <c r="AU40">
         <v>0.5</v>
       </c>
+      <c r="AW40" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="41" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>140</v>
       </c>
@@ -7240,8 +7326,7 @@
         <v>172.51490514026949</v>
       </c>
       <c r="W41" s="6">
-        <f t="shared" si="3"/>
-        <v>126.855553995847</v>
+        <v>171.8202545199316</v>
       </c>
       <c r="X41" s="6">
         <f t="shared" si="4"/>
@@ -7251,8 +7336,8 @@
         <v>0.8</v>
       </c>
       <c r="Z41" s="6">
-        <f t="shared" si="2"/>
-        <v>156.3847963141107</v>
+        <f>W41</f>
+        <v>171.8202545199316</v>
       </c>
       <c r="AA41" s="6">
         <v>40.633259071626938</v>
@@ -7317,8 +7402,11 @@
       <c r="AU41">
         <v>0.5</v>
       </c>
+      <c r="AW41" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="42" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>142</v>
       </c>
@@ -7386,8 +7474,7 @@
         <v>149.57196905597809</v>
       </c>
       <c r="W42" s="6">
-        <f t="shared" si="3"/>
-        <v>158.86574298419873</v>
+        <v>198.72214236512679</v>
       </c>
       <c r="X42" s="6">
         <f t="shared" si="4"/>
@@ -7397,8 +7484,8 @@
         <v>0.8</v>
       </c>
       <c r="Z42" s="6">
-        <f t="shared" si="2"/>
-        <v>185.04025902756752</v>
+        <f>W42</f>
+        <v>198.72214236512679</v>
       </c>
       <c r="AA42" s="6">
         <v>39.30265205847347</v>
@@ -7463,8 +7550,11 @@
       <c r="AU42">
         <v>0.5</v>
       </c>
+      <c r="AW42" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="43" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>144</v>
       </c>
@@ -7532,8 +7622,7 @@
         <v>133.16678784249231</v>
       </c>
       <c r="W43" s="6">
-        <f t="shared" si="3"/>
-        <v>159.91922490811703</v>
+        <v>192.09633796783118</v>
       </c>
       <c r="X43" s="6">
         <f t="shared" si="4"/>
@@ -7543,8 +7632,8 @@
         <v>0.8</v>
       </c>
       <c r="Z43" s="6">
-        <f t="shared" si="2"/>
-        <v>181.05059590731952</v>
+        <f>W43</f>
+        <v>192.09633796783118</v>
       </c>
       <c r="AA43" s="6">
         <v>80.842005676442767</v>
@@ -7609,8 +7698,11 @@
       <c r="AU43">
         <v>0.5</v>
       </c>
+      <c r="AW43" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="44" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>146</v>
       </c>
@@ -7678,8 +7770,7 @@
         <v>221.3471308699809</v>
       </c>
       <c r="W44" s="6">
-        <f t="shared" si="3"/>
-        <v>158.07755498044571</v>
+        <v>195.10524025063538</v>
       </c>
       <c r="X44" s="6">
         <f t="shared" si="4"/>
@@ -7689,8 +7780,8 @@
         <v>0.8</v>
       </c>
       <c r="Z44" s="6">
-        <f t="shared" si="2"/>
-        <v>182.39439637122001</v>
+        <f>W44</f>
+        <v>195.10524025063538</v>
       </c>
       <c r="AA44" s="6">
         <v>24.194769127475819</v>
@@ -7755,8 +7846,11 @@
       <c r="AU44">
         <v>0.5</v>
       </c>
+      <c r="AW44" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="45" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>148</v>
       </c>
@@ -7824,8 +7918,7 @@
         <v>155.7833631217363</v>
       </c>
       <c r="W45" s="6">
-        <f t="shared" si="3"/>
-        <v>146.97805890264138</v>
+        <v>179.038426011581</v>
       </c>
       <c r="X45" s="6">
         <f t="shared" si="4"/>
@@ -7835,8 +7928,8 @@
         <v>0.8</v>
       </c>
       <c r="Z45" s="6">
-        <f t="shared" si="2"/>
-        <v>168.03276043824428</v>
+        <f>W45</f>
+        <v>179.038426011581</v>
       </c>
       <c r="AA45" s="6">
         <v>61.087984862819297</v>
@@ -7901,8 +7994,11 @@
       <c r="AU45">
         <v>0.5</v>
       </c>
+      <c r="AW45" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="46" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>150</v>
       </c>
@@ -7970,8 +8066,7 @@
         <v>164.052579899726</v>
       </c>
       <c r="W46" s="6">
-        <f t="shared" si="3"/>
-        <v>146.49845108251611</v>
+        <v>186.07567024012963</v>
       </c>
       <c r="X46" s="6">
         <f t="shared" si="4"/>
@@ -7981,8 +8076,8 @@
         <v>0.8</v>
       </c>
       <c r="Z46" s="6">
-        <f t="shared" si="2"/>
-        <v>172.48962373943641</v>
+        <f>W46</f>
+        <v>186.07567024012963</v>
       </c>
       <c r="AA46" s="6">
         <v>84.135563219092376</v>
@@ -8047,8 +8142,11 @@
       <c r="AU46">
         <v>0.5</v>
       </c>
+      <c r="AW46" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="47" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>153</v>
       </c>
@@ -8116,8 +8214,7 @@
         <v>99.325228953966871</v>
       </c>
       <c r="W47" s="6">
-        <f t="shared" si="3"/>
-        <v>139.2557298153406</v>
+        <v>182.26123166696325</v>
       </c>
       <c r="X47" s="6">
         <f t="shared" si="4"/>
@@ -8127,8 +8224,8 @@
         <v>0.8</v>
       </c>
       <c r="Z47" s="6">
-        <f t="shared" si="2"/>
-        <v>167.49832612741639</v>
+        <f>W47</f>
+        <v>182.26123166696325</v>
       </c>
       <c r="AA47" s="6">
         <v>58.619647816400651</v>
@@ -8193,8 +8290,11 @@
       <c r="AU47">
         <v>0.5</v>
       </c>
+      <c r="AW47" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="48" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>155</v>
       </c>
@@ -8262,8 +8362,7 @@
         <v>148.77071559239991</v>
       </c>
       <c r="W48" s="6">
-        <f t="shared" si="3"/>
-        <v>161.82337996397109</v>
+        <v>203.99130386920152</v>
       </c>
       <c r="X48" s="6">
         <f t="shared" si="4"/>
@@ -8273,8 +8372,8 @@
         <v>0.8</v>
       </c>
       <c r="Z48" s="6">
-        <f t="shared" si="2"/>
-        <v>189.51592163649244</v>
+        <f>W48</f>
+        <v>203.99130386920152</v>
       </c>
       <c r="AA48" s="6">
         <v>22.617572557756279</v>
@@ -8339,8 +8438,11 @@
       <c r="AU48">
         <v>0.5</v>
       </c>
+      <c r="AW48" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="49" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>157</v>
       </c>
@@ -8408,8 +8510,7 @@
         <v>204.78768798639069</v>
       </c>
       <c r="W49" s="6">
-        <f t="shared" si="3"/>
-        <v>153.42526220720174</v>
+        <v>196.23667863334515</v>
       </c>
       <c r="X49" s="6">
         <f t="shared" si="4"/>
@@ -8419,8 +8520,8 @@
         <v>0.8</v>
       </c>
       <c r="Z49" s="6">
-        <f t="shared" si="2"/>
-        <v>181.54039863424285</v>
+        <f>W49</f>
+        <v>196.23667863334515</v>
       </c>
       <c r="AA49" s="6">
         <v>20.53254799035615</v>
@@ -8485,8 +8586,11 @@
       <c r="AU49">
         <v>0.5</v>
       </c>
+      <c r="AW49" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="50" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>159</v>
       </c>
@@ -8554,8 +8658,7 @@
         <v>190.43811259180069</v>
       </c>
       <c r="W50" s="6">
-        <f t="shared" si="3"/>
-        <v>154.86820397327392</v>
+        <v>201.5919979382004</v>
       </c>
       <c r="X50" s="6">
         <f t="shared" si="4"/>
@@ -8565,8 +8668,8 @@
         <v>0.8</v>
       </c>
       <c r="Z50" s="6">
-        <f t="shared" si="2"/>
-        <v>185.55267908236354</v>
+        <f>W50</f>
+        <v>201.5919979382004</v>
       </c>
       <c r="AA50" s="6">
         <v>46.80288094729454</v>
@@ -8631,8 +8734,11 @@
       <c r="AU50">
         <v>0.5</v>
       </c>
+      <c r="AW50" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="51" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>161</v>
       </c>
@@ -8700,8 +8806,7 @@
         <v>107.06784829963</v>
       </c>
       <c r="W51" s="6">
-        <f t="shared" si="3"/>
-        <v>154.63045637388859</v>
+        <v>196.59633483927811</v>
       </c>
       <c r="X51" s="6">
         <f t="shared" si="4"/>
@@ -8711,8 +8816,8 @@
         <v>0.8</v>
       </c>
       <c r="Z51" s="6">
-        <f t="shared" si="2"/>
-        <v>182.19031065646132</v>
+        <f>W51</f>
+        <v>196.59633483927811</v>
       </c>
       <c r="AA51" s="6">
         <v>80.475783562730797</v>
@@ -8777,8 +8882,11 @@
       <c r="AU51">
         <v>0.5</v>
       </c>
+      <c r="AW51" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="52" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>163</v>
       </c>
@@ -8846,8 +8954,7 @@
         <v>184.50550138950351</v>
       </c>
       <c r="W52" s="6">
-        <f t="shared" si="3"/>
-        <v>152.23049028136302</v>
+        <v>190.63442664306874</v>
       </c>
       <c r="X52" s="6">
         <f t="shared" si="4"/>
@@ -8857,8 +8964,8 @@
         <v>0.8</v>
       </c>
       <c r="Z52" s="6">
-        <f t="shared" si="2"/>
-        <v>177.45114402935275</v>
+        <f>W52</f>
+        <v>190.63442664306874</v>
       </c>
       <c r="AA52" s="6">
         <v>77.594836268196659</v>
@@ -8923,8 +9030,11 @@
       <c r="AU52">
         <v>0.5</v>
       </c>
+      <c r="AW52" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="53" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>165</v>
       </c>
@@ -8992,8 +9102,7 @@
         <v>175.4236738328473</v>
       </c>
       <c r="W53" s="6">
-        <f t="shared" si="3"/>
-        <v>160.10378696264524</v>
+        <v>197.90306788510551</v>
       </c>
       <c r="X53" s="6">
         <f t="shared" si="4"/>
@@ -9003,8 +9112,8 @@
         <v>0.8</v>
       </c>
       <c r="Z53" s="6">
-        <f t="shared" si="2"/>
-        <v>184.92735106528153</v>
+        <f>W53</f>
+        <v>197.90306788510551</v>
       </c>
       <c r="AA53" s="6">
         <v>37.246925260170293</v>
@@ -9069,8 +9178,11 @@
       <c r="AU53">
         <v>0.5</v>
       </c>
+      <c r="AW53" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="54" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>167</v>
       </c>
@@ -9138,8 +9250,7 @@
         <v>213.494826463284</v>
       </c>
       <c r="W54" s="6">
-        <f t="shared" si="3"/>
-        <v>145.62584207524196</v>
+        <v>186.62184926048724</v>
       </c>
       <c r="X54" s="6">
         <f t="shared" si="4"/>
@@ -9149,8 +9260,8 @@
         <v>0.8</v>
       </c>
       <c r="Z54" s="6">
-        <f t="shared" si="2"/>
-        <v>172.54876196894753</v>
+        <f>W54</f>
+        <v>186.62184926048724</v>
       </c>
       <c r="AA54" s="6">
         <v>24.71724600970489</v>
@@ -9215,8 +9326,11 @@
       <c r="AU54">
         <v>0.5</v>
       </c>
+      <c r="AW54" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="55" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>170</v>
       </c>
@@ -9284,8 +9398,7 @@
         <v>139.13817762513639</v>
       </c>
       <c r="W55" s="6">
-        <f t="shared" si="3"/>
-        <v>151.86279578429091</v>
+        <v>191.28353897506068</v>
       </c>
       <c r="X55" s="6">
         <f t="shared" si="4"/>
@@ -9295,8 +9408,8 @@
         <v>0.8</v>
       </c>
       <c r="Z55" s="6">
-        <f t="shared" si="2"/>
-        <v>177.75120746008486</v>
+        <f>W55</f>
+        <v>191.28353897506068</v>
       </c>
       <c r="AA55" s="6">
         <v>54.176152836695451</v>
@@ -9361,8 +9474,11 @@
       <c r="AU55">
         <v>0.5</v>
       </c>
+      <c r="AW55" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="56" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>172</v>
       </c>
@@ -9430,8 +9546,7 @@
         <v>156.51459686196179</v>
       </c>
       <c r="W56" s="6">
-        <f t="shared" si="3"/>
-        <v>151.00319539342308</v>
+        <v>185.76313024000677</v>
       </c>
       <c r="X56" s="6">
         <f t="shared" si="4"/>
@@ -9441,8 +9556,8 @@
         <v>0.8</v>
       </c>
       <c r="Z56" s="6">
-        <f t="shared" si="2"/>
-        <v>173.83075850600389</v>
+        <f>W56</f>
+        <v>185.76313024000677</v>
       </c>
       <c r="AA56" s="6">
         <v>23.550218207342748</v>
@@ -9507,8 +9622,11 @@
       <c r="AU56">
         <v>0.5</v>
       </c>
+      <c r="AW56" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="57" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>174</v>
       </c>
@@ -9576,8 +9694,7 @@
         <v>182.41111699026081</v>
       </c>
       <c r="W57" s="6">
-        <f t="shared" si="3"/>
-        <v>150.20910420062137</v>
+        <v>186.79555680803142</v>
       </c>
       <c r="X57" s="6">
         <f t="shared" si="4"/>
@@ -9587,8 +9704,8 @@
         <v>0.8</v>
       </c>
       <c r="Z57" s="6">
-        <f t="shared" si="2"/>
-        <v>174.23617903972098</v>
+        <f>W57</f>
+        <v>186.79555680803142</v>
       </c>
       <c r="AA57" s="6">
         <v>43.177282021546063</v>
@@ -9653,8 +9770,11 @@
       <c r="AU57">
         <v>0.5</v>
       </c>
+      <c r="AW57" s="7">
+        <v>0.9</v>
+      </c>
     </row>
-    <row r="58" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>176</v>
       </c>
@@ -9722,8 +9842,7 @@
         <v>129.45376435382059</v>
       </c>
       <c r="W58" s="6">
-        <f t="shared" si="3"/>
-        <v>154.61894273939834</v>
+        <v>163.32740587284957</v>
       </c>
       <c r="X58" s="6">
         <f t="shared" si="4"/>
@@ -9733,8 +9852,8 @@
         <v>0.8</v>
       </c>
       <c r="Z58" s="6">
-        <f t="shared" si="2"/>
-        <v>183.54853141115373</v>
+        <f>W58</f>
+        <v>163.32740587284957</v>
       </c>
       <c r="AA58" s="6">
         <v>30.945463423566391</v>
@@ -9799,8 +9918,11 @@
       <c r="AU58">
         <v>0.5</v>
       </c>
+      <c r="AW58" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="59" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>179</v>
       </c>
@@ -9868,8 +9990,7 @@
         <v>142.0250161267177</v>
       </c>
       <c r="W59" s="6">
-        <f t="shared" si="3"/>
-        <v>154.4507231677926</v>
+        <v>161.5672843806309</v>
       </c>
       <c r="X59" s="6">
         <f t="shared" si="4"/>
@@ -9879,8 +10000,8 @@
         <v>0.8</v>
       </c>
       <c r="Z59" s="6">
-        <f t="shared" si="2"/>
-        <v>178.09200010607927</v>
+        <f>W59</f>
+        <v>161.5672843806309</v>
       </c>
       <c r="AA59" s="6">
         <v>73.620105594042798</v>
@@ -9945,8 +10066,11 @@
       <c r="AU59">
         <v>0.5</v>
       </c>
+      <c r="AW59" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="60" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>181</v>
       </c>
@@ -10014,8 +10138,7 @@
         <v>189.92597612523241</v>
       </c>
       <c r="W60" s="6">
-        <f t="shared" si="3"/>
-        <v>146.78916537959594</v>
+        <v>156.3758318070575</v>
       </c>
       <c r="X60" s="6">
         <f t="shared" si="4"/>
@@ -10025,8 +10148,8 @@
         <v>0.8</v>
       </c>
       <c r="Z60" s="6">
-        <f t="shared" si="2"/>
-        <v>178.63615287093282</v>
+        <f>W60</f>
+        <v>156.3758318070575</v>
       </c>
       <c r="AA60" s="6">
         <v>85.517441328165532</v>
@@ -10091,8 +10214,11 @@
       <c r="AU60">
         <v>0.5</v>
       </c>
+      <c r="AW60" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="61" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>183</v>
       </c>
@@ -10160,8 +10286,7 @@
         <v>163.91445039189421</v>
       </c>
       <c r="W61" s="6">
-        <f t="shared" si="3"/>
-        <v>146.49467952167473</v>
+        <v>152.10720085580056</v>
       </c>
       <c r="X61" s="6">
         <f t="shared" si="4"/>
@@ -10171,8 +10296,8 @@
         <v>0.8</v>
       </c>
       <c r="Z61" s="6">
-        <f t="shared" si="2"/>
-        <v>165.13952317772916</v>
+        <f>W61</f>
+        <v>152.10720085580056</v>
       </c>
       <c r="AA61" s="6">
         <v>34.719992675557727</v>
@@ -10237,8 +10362,11 @@
       <c r="AU61">
         <v>0.5</v>
       </c>
+      <c r="AW61" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="62" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>186</v>
       </c>
@@ -10306,8 +10434,7 @@
         <v>135.02638618447239</v>
       </c>
       <c r="W62" s="6">
-        <f t="shared" si="3"/>
-        <v>143.10909970517969</v>
+        <v>149.62686266129109</v>
       </c>
       <c r="X62" s="6">
         <f t="shared" si="4"/>
@@ -10317,8 +10444,8 @@
         <v>0.8</v>
       </c>
       <c r="Z62" s="6">
-        <f t="shared" si="2"/>
-        <v>164.76116373654929</v>
+        <f>W62</f>
+        <v>149.62686266129109</v>
       </c>
       <c r="AA62" s="6">
         <v>56.202581865901671</v>
@@ -10383,8 +10510,11 @@
       <c r="AU62">
         <v>0.5</v>
       </c>
+      <c r="AW62" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="63" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>188</v>
       </c>
@@ -10452,8 +10582,7 @@
         <v>162.06416300192359</v>
       </c>
       <c r="W63" s="6">
-        <f t="shared" si="3"/>
-        <v>160.42000405959698</v>
+        <v>168.7620619614402</v>
       </c>
       <c r="X63" s="6">
         <f t="shared" si="4"/>
@@ -10463,8 +10592,8 @@
         <v>0.8</v>
       </c>
       <c r="Z63" s="6">
-        <f t="shared" si="2"/>
-        <v>188.13239143243635</v>
+        <f>W63</f>
+        <v>168.7620619614402</v>
       </c>
       <c r="AA63" s="6">
         <v>49.991454817346721</v>
@@ -10529,8 +10658,11 @@
       <c r="AU63">
         <v>0.5</v>
       </c>
+      <c r="AW63" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="64" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>190</v>
       </c>
@@ -10598,8 +10730,7 @@
         <v>94.967294140951708</v>
       </c>
       <c r="W64" s="6">
-        <f t="shared" si="3"/>
-        <v>143.93246241652378</v>
+        <v>149.96684985419955</v>
       </c>
       <c r="X64" s="6">
         <f t="shared" si="4"/>
@@ -10609,8 +10740,8 @@
         <v>0.8</v>
       </c>
       <c r="Z64" s="6">
-        <f t="shared" si="2"/>
-        <v>163.97874886027012</v>
+        <f>W64</f>
+        <v>149.96684985419955</v>
       </c>
       <c r="AA64" s="6">
         <v>60.895107882931001</v>
@@ -10675,8 +10806,11 @@
       <c r="AU64">
         <v>0.5</v>
       </c>
+      <c r="AW64" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="65" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>192</v>
       </c>
@@ -10744,8 +10878,7 @@
         <v>126.2178504170151</v>
       </c>
       <c r="W65" s="6">
-        <f t="shared" si="3"/>
-        <v>143.44493915032217</v>
+        <v>152.26920744094528</v>
       </c>
       <c r="X65" s="6">
         <f t="shared" si="4"/>
@@ -10755,8 +10888,8 @@
         <v>0.8</v>
       </c>
       <c r="Z65" s="6">
-        <f t="shared" si="2"/>
-        <v>172.7592335401487</v>
+        <f>W65</f>
+        <v>152.26920744094528</v>
       </c>
       <c r="AA65" s="6">
         <v>80.998260444959868</v>
@@ -10821,8 +10954,11 @@
       <c r="AU65">
         <v>0.5</v>
       </c>
+      <c r="AW65" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="66" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>194</v>
       </c>
@@ -10890,8 +11026,7 @@
         <v>118.23539731849451</v>
       </c>
       <c r="W66" s="6">
-        <f t="shared" si="3"/>
-        <v>143.4172393523113</v>
+        <v>152.9469633052199</v>
       </c>
       <c r="X66" s="6">
         <f t="shared" si="4"/>
@@ -10901,8 +11036,8 @@
         <v>0.8</v>
       </c>
       <c r="Z66" s="6">
-        <f t="shared" si="2"/>
-        <v>175.07506345838434</v>
+        <f>W66</f>
+        <v>152.9469633052199</v>
       </c>
       <c r="AA66" s="6">
         <v>15.652027954954679</v>
@@ -10967,8 +11102,11 @@
       <c r="AU66">
         <v>0.5</v>
       </c>
+      <c r="AW66" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="67" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>196</v>
       </c>
@@ -11036,8 +11174,7 @@
         <v>150.85728970589119</v>
       </c>
       <c r="W67" s="6">
-        <f t="shared" si="3"/>
-        <v>142.84734144566758</v>
+        <v>150.22105179915368</v>
       </c>
       <c r="X67" s="6">
         <f t="shared" si="4"/>
@@ -11047,8 +11184,8 @@
         <v>0.8</v>
       </c>
       <c r="Z67" s="6">
-        <f t="shared" si="2"/>
-        <v>167.34287001851206</v>
+        <f>W67</f>
+        <v>150.22105179915368</v>
       </c>
       <c r="AA67" s="6">
         <v>58.375499740592673</v>
@@ -11113,8 +11250,11 @@
       <c r="AU67">
         <v>0.5</v>
       </c>
+      <c r="AW67" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="68" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>198</v>
       </c>
@@ -11182,8 +11322,7 @@
         <v>208.7079739489127</v>
       </c>
       <c r="W68" s="6">
-        <f t="shared" si="3"/>
-        <v>156.56908980545268</v>
+        <v>162.86018342496118</v>
       </c>
       <c r="X68" s="6">
         <f t="shared" si="4"/>
@@ -11193,8 +11332,8 @@
         <v>0.8</v>
       </c>
       <c r="Z68" s="6">
-        <f t="shared" ref="Z68:Z100" si="5">NORMINV(Y68,W68,X68)</f>
-        <v>177.46815637080192</v>
+        <f>W68</f>
+        <v>162.86018342496118</v>
       </c>
       <c r="AA68" s="6">
         <v>58.348643452253803</v>
@@ -11259,8 +11398,11 @@
       <c r="AU68">
         <v>0.5</v>
       </c>
+      <c r="AW68" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="69" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>200</v>
       </c>
@@ -11328,8 +11470,7 @@
         <v>139.01314484101019</v>
       </c>
       <c r="W69" s="6">
-        <f t="shared" ref="W69:W100" si="6">AVERAGE(K69:V69)</f>
-        <v>157.64837864153375</v>
+        <v>166.28622283038322</v>
       </c>
       <c r="X69" s="6">
         <f t="shared" ref="X69:X100" si="7">_xlfn.STDEV.S(K69:V69)</f>
@@ -11339,8 +11480,8 @@
         <v>0.8</v>
       </c>
       <c r="Z69" s="6">
-        <f t="shared" si="5"/>
-        <v>186.34337057808392</v>
+        <f>W69</f>
+        <v>166.28622283038322</v>
       </c>
       <c r="AA69" s="6">
         <v>12.67830439161351</v>
@@ -11405,8 +11546,11 @@
       <c r="AU69">
         <v>0.5</v>
       </c>
+      <c r="AW69" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="70" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>202</v>
       </c>
@@ -11474,8 +11618,7 @@
         <v>119.5975247959723</v>
       </c>
       <c r="W70" s="6">
-        <f t="shared" si="6"/>
-        <v>139.59894469408027</v>
+        <v>146.52940748746974</v>
       </c>
       <c r="X70" s="6">
         <f t="shared" si="7"/>
@@ -11485,8 +11628,8 @@
         <v>0.8</v>
       </c>
       <c r="Z70" s="6">
-        <f t="shared" si="5"/>
-        <v>162.62200109854655</v>
+        <f>W70</f>
+        <v>146.52940748746974</v>
       </c>
       <c r="AA70" s="6">
         <v>12.96639912106693</v>
@@ -11551,8 +11694,11 @@
       <c r="AU70">
         <v>0.5</v>
       </c>
+      <c r="AW70" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="71" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>204</v>
       </c>
@@ -11620,8 +11766,7 @@
         <v>158.80311290529789</v>
       </c>
       <c r="W71" s="6">
-        <f t="shared" si="6"/>
-        <v>141.32583070604596</v>
+        <v>148.42374788167882</v>
       </c>
       <c r="X71" s="6">
         <f t="shared" si="7"/>
@@ -11631,8 +11776,8 @@
         <v>0.8</v>
       </c>
       <c r="Z71" s="6">
-        <f t="shared" si="5"/>
-        <v>164.90517199400389</v>
+        <f>W71</f>
+        <v>148.42374788167882</v>
       </c>
       <c r="AA71" s="6">
         <v>29.880977813043611</v>
@@ -11697,8 +11842,11 @@
       <c r="AU71">
         <v>0.5</v>
       </c>
+      <c r="AW71" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="72" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>206</v>
       </c>
@@ -11766,8 +11914,7 @@
         <v>209.49077603872871</v>
       </c>
       <c r="W72" s="6">
-        <f t="shared" si="6"/>
-        <v>151.27954251638585</v>
+        <v>159.55675745533225</v>
       </c>
       <c r="X72" s="6">
         <f t="shared" si="7"/>
@@ -11777,8 +11924,8 @@
         <v>0.8</v>
       </c>
       <c r="Z72" s="6">
-        <f t="shared" si="5"/>
-        <v>178.77652101441961</v>
+        <f>W72</f>
+        <v>159.55675745533225</v>
       </c>
       <c r="AA72" s="6">
         <v>51.058381908627581</v>
@@ -11843,8 +11990,11 @@
       <c r="AU72">
         <v>0.5</v>
       </c>
+      <c r="AW72" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="73" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>208</v>
       </c>
@@ -11912,8 +12062,7 @@
         <v>172.00113158323799</v>
       </c>
       <c r="W73" s="6">
-        <f t="shared" si="6"/>
-        <v>153.26676286022121</v>
+        <v>160.20311565862482</v>
       </c>
       <c r="X73" s="6">
         <f t="shared" si="7"/>
@@ -11923,8 +12072,8 @@
         <v>0.8</v>
       </c>
       <c r="Z73" s="6">
-        <f t="shared" si="5"/>
-        <v>176.30938591149098</v>
+        <f>W73</f>
+        <v>160.20311565862482</v>
       </c>
       <c r="AA73" s="6">
         <v>88.066347239600816</v>
@@ -11989,8 +12138,11 @@
       <c r="AU73">
         <v>0.5</v>
       </c>
+      <c r="AW73" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="74" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>210</v>
       </c>
@@ -12058,8 +12210,7 @@
         <v>96.283787721768022</v>
       </c>
       <c r="W74" s="6">
-        <f t="shared" si="6"/>
-        <v>132.99458070505355</v>
+        <v>139.1711439534152</v>
       </c>
       <c r="X74" s="6">
         <f t="shared" si="7"/>
@@ -12069,8 +12220,8 @@
         <v>0.8</v>
       </c>
       <c r="Z74" s="6">
-        <f t="shared" si="5"/>
-        <v>153.51317640235999</v>
+        <f>W74</f>
+        <v>139.1711439534152</v>
       </c>
       <c r="AA74" s="6">
         <v>88.537553025910213</v>
@@ -12135,8 +12286,11 @@
       <c r="AU74">
         <v>0.5</v>
       </c>
+      <c r="AW74" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="75" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>212</v>
       </c>
@@ -12204,8 +12358,7 @@
         <v>189.79289431299549</v>
       </c>
       <c r="W75" s="6">
-        <f t="shared" si="6"/>
-        <v>154.61379840999143</v>
+        <v>162.63451446856652</v>
       </c>
       <c r="X75" s="6">
         <f t="shared" si="7"/>
@@ -12215,8 +12368,8 @@
         <v>0.8</v>
       </c>
       <c r="Z75" s="6">
-        <f t="shared" si="5"/>
-        <v>181.25868544364229</v>
+        <f>W75</f>
+        <v>162.63451446856652</v>
       </c>
       <c r="AA75" s="6">
         <v>18.716086306344799</v>
@@ -12281,8 +12434,11 @@
       <c r="AU75">
         <v>0.5</v>
       </c>
+      <c r="AW75" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="76" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>214</v>
       </c>
@@ -12350,8 +12506,7 @@
         <v>161.43725967267531</v>
       </c>
       <c r="W76" s="6">
-        <f t="shared" si="6"/>
-        <v>154.64345362161112</v>
+        <v>162.96893093512614</v>
       </c>
       <c r="X76" s="6">
         <f t="shared" si="7"/>
@@ -12361,8 +12516,8 @@
         <v>0.8</v>
       </c>
       <c r="Z76" s="6">
-        <f t="shared" si="5"/>
-        <v>182.30076013885989</v>
+        <f>W76</f>
+        <v>162.96893093512614</v>
       </c>
       <c r="AA76" s="6">
         <v>52.381664479506817</v>
@@ -12427,8 +12582,11 @@
       <c r="AU76">
         <v>0.5</v>
       </c>
+      <c r="AW76" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="77" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>216</v>
       </c>
@@ -12496,8 +12654,7 @@
         <v>152.01304146685291</v>
       </c>
       <c r="W77" s="6">
-        <f t="shared" si="6"/>
-        <v>141.99117723946983</v>
+        <v>145.77383916414826</v>
       </c>
       <c r="X77" s="6">
         <f t="shared" si="7"/>
@@ -12507,8 +12664,8 @@
         <v>0.8</v>
       </c>
       <c r="Z77" s="6">
-        <f t="shared" si="5"/>
-        <v>154.55721235821625</v>
+        <f>W77</f>
+        <v>145.77383916414826</v>
       </c>
       <c r="AA77" s="6">
         <v>25.693838312936801</v>
@@ -12573,8 +12730,11 @@
       <c r="AU77">
         <v>0.5</v>
       </c>
+      <c r="AW77" s="7">
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="78" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>219</v>
       </c>
@@ -12642,7 +12802,6 @@
         <v>142.34080405585701</v>
       </c>
       <c r="W78" s="6">
-        <f t="shared" si="6"/>
         <v>148.52124972221645</v>
       </c>
       <c r="X78" s="6">
@@ -12653,8 +12812,8 @@
         <v>0.8</v>
       </c>
       <c r="Z78" s="6">
-        <f t="shared" si="5"/>
-        <v>179.32706867790114</v>
+        <f>W78</f>
+        <v>148.52124972221645</v>
       </c>
       <c r="AA78" s="6">
         <v>44.886318552201907</v>
@@ -12719,8 +12878,11 @@
       <c r="AU78">
         <v>0.5</v>
       </c>
+      <c r="AW78" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="79" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>222</v>
       </c>
@@ -12788,7 +12950,6 @@
         <v>184.27971932978829</v>
       </c>
       <c r="W79" s="6">
-        <f t="shared" si="6"/>
         <v>153.14875023832428</v>
       </c>
       <c r="X79" s="6">
@@ -12799,8 +12960,8 @@
         <v>0.8</v>
       </c>
       <c r="Z79" s="6">
-        <f t="shared" si="5"/>
-        <v>186.47241984983609</v>
+        <f>W79</f>
+        <v>153.14875023832428</v>
       </c>
       <c r="AA79" s="6">
         <v>37.205420087282938</v>
@@ -12865,8 +13026,11 @@
       <c r="AU79">
         <v>0.5</v>
       </c>
+      <c r="AW79" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="80" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>225</v>
       </c>
@@ -12934,7 +13098,6 @@
         <v>131.57379650365331</v>
       </c>
       <c r="W80" s="6">
-        <f t="shared" si="6"/>
         <v>140.66451437101932</v>
       </c>
       <c r="X80" s="6">
@@ -12945,8 +13108,8 @@
         <v>0.8</v>
       </c>
       <c r="Z80" s="6">
-        <f t="shared" si="5"/>
-        <v>160.26771167898923</v>
+        <f>W80</f>
+        <v>140.66451437101932</v>
       </c>
       <c r="AA80" s="6">
         <v>19.543748283333841</v>
@@ -13011,8 +13174,11 @@
       <c r="AU80">
         <v>0.5</v>
       </c>
+      <c r="AW80" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="81" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>227</v>
       </c>
@@ -13080,7 +13246,6 @@
         <v>147.174177224224</v>
       </c>
       <c r="W81" s="6">
-        <f t="shared" si="6"/>
         <v>143.77028530034295</v>
       </c>
       <c r="X81" s="6">
@@ -13091,8 +13256,8 @@
         <v>0.8</v>
       </c>
       <c r="Z81" s="6">
-        <f t="shared" si="5"/>
-        <v>160.71372553026066</v>
+        <f>W81</f>
+        <v>143.77028530034295</v>
       </c>
       <c r="AA81" s="6">
         <v>73.590807824945827</v>
@@ -13157,8 +13322,11 @@
       <c r="AU81">
         <v>0.5</v>
       </c>
+      <c r="AW81" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="82" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>229</v>
       </c>
@@ -13226,7 +13394,6 @@
         <v>195.4147993877996</v>
       </c>
       <c r="W82" s="6">
-        <f t="shared" si="6"/>
         <v>169.47236967225763</v>
       </c>
       <c r="X82" s="6">
@@ -13237,8 +13404,8 @@
         <v>0.8</v>
       </c>
       <c r="Z82" s="6">
-        <f t="shared" si="5"/>
-        <v>193.14075064914189</v>
+        <f>W82</f>
+        <v>169.47236967225763</v>
       </c>
       <c r="AA82" s="6">
         <v>86.381725516525762</v>
@@ -13303,8 +13470,11 @@
       <c r="AU82">
         <v>0.5</v>
       </c>
+      <c r="AW82" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="83" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>231</v>
       </c>
@@ -13372,8 +13542,7 @@
         <v>121.2176304456079</v>
       </c>
       <c r="W83" s="6">
-        <f t="shared" si="6"/>
-        <v>150.00363229446521</v>
+        <v>150.0036322944652</v>
       </c>
       <c r="X83" s="6">
         <f t="shared" si="7"/>
@@ -13383,8 +13552,8 @@
         <v>0.8</v>
       </c>
       <c r="Z83" s="6">
-        <f t="shared" si="5"/>
-        <v>168.24810915691387</v>
+        <f>W83</f>
+        <v>150.0036322944652</v>
       </c>
       <c r="AA83" s="6">
         <v>19.866023743400369</v>
@@ -13449,8 +13618,11 @@
       <c r="AU83">
         <v>0.5</v>
       </c>
+      <c r="AW83" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="84" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>233</v>
       </c>
@@ -13518,7 +13690,6 @@
         <v>146.16968580085091</v>
       </c>
       <c r="W84" s="6">
-        <f t="shared" si="6"/>
         <v>161.0622153215445</v>
       </c>
       <c r="X84" s="6">
@@ -13529,8 +13700,8 @@
         <v>0.8</v>
       </c>
       <c r="Z84" s="6">
-        <f t="shared" si="5"/>
-        <v>187.85760809036103</v>
+        <f>W84</f>
+        <v>161.0622153215445</v>
       </c>
       <c r="AA84" s="6">
         <v>34.680928983428451</v>
@@ -13595,8 +13766,11 @@
       <c r="AU84">
         <v>0.5</v>
       </c>
+      <c r="AW84" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="85" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>235</v>
       </c>
@@ -13664,8 +13838,7 @@
         <v>162.61613533642961</v>
       </c>
       <c r="W85" s="6">
-        <f t="shared" si="6"/>
-        <v>149.03922400790179</v>
+        <v>149.0392240079018</v>
       </c>
       <c r="X85" s="6">
         <f t="shared" si="7"/>
@@ -13675,8 +13848,8 @@
         <v>0.8</v>
       </c>
       <c r="Z85" s="6">
-        <f t="shared" si="5"/>
-        <v>167.93625305243563</v>
+        <f>W85</f>
+        <v>149.0392240079018</v>
       </c>
       <c r="AA85" s="6">
         <v>49.356669820245983</v>
@@ -13741,8 +13914,11 @@
       <c r="AU85">
         <v>0.5</v>
       </c>
+      <c r="AW85" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="86" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>237</v>
       </c>
@@ -13810,7 +13986,6 @@
         <v>115.6187128493912</v>
       </c>
       <c r="W86" s="6">
-        <f t="shared" si="6"/>
         <v>148.40689213215228</v>
       </c>
       <c r="X86" s="6">
@@ -13821,8 +13996,8 @@
         <v>0.8</v>
       </c>
       <c r="Z86" s="6">
-        <f t="shared" si="5"/>
-        <v>172.14445598964036</v>
+        <f>W86</f>
+        <v>148.40689213215228</v>
       </c>
       <c r="AA86" s="6">
         <v>68.295236060670803</v>
@@ -13887,8 +14062,11 @@
       <c r="AU86">
         <v>0.5</v>
       </c>
+      <c r="AW86" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="87" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>239</v>
       </c>
@@ -13956,7 +14134,6 @@
         <v>145.75048832411991</v>
       </c>
       <c r="W87" s="6">
-        <f t="shared" si="6"/>
         <v>144.452238638587</v>
       </c>
       <c r="X87" s="6">
@@ -13967,8 +14144,8 @@
         <v>0.8</v>
       </c>
       <c r="Z87" s="6">
-        <f t="shared" si="5"/>
-        <v>162.60233321090237</v>
+        <f>W87</f>
+        <v>144.452238638587</v>
       </c>
       <c r="AA87" s="6">
         <v>63.683278908658103</v>
@@ -14033,8 +14210,11 @@
       <c r="AU87">
         <v>0.5</v>
       </c>
+      <c r="AW87" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="88" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>241</v>
       </c>
@@ -14102,7 +14282,6 @@
         <v>132.2591234988067</v>
       </c>
       <c r="W88" s="6">
-        <f t="shared" si="6"/>
         <v>144.53525276749133</v>
       </c>
       <c r="X88" s="6">
@@ -14113,8 +14292,8 @@
         <v>0.8</v>
       </c>
       <c r="Z88" s="6">
-        <f t="shared" si="5"/>
-        <v>164.75754505506228</v>
+        <f>W88</f>
+        <v>144.53525276749133</v>
       </c>
       <c r="AA88" s="6">
         <v>71.613208410901208</v>
@@ -14179,8 +14358,11 @@
       <c r="AU88">
         <v>0.5</v>
       </c>
+      <c r="AW88" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="89" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>243</v>
       </c>
@@ -14248,7 +14430,6 @@
         <v>154.34688445238859</v>
       </c>
       <c r="W89" s="6">
-        <f t="shared" si="6"/>
         <v>142.22395103970482</v>
       </c>
       <c r="X89" s="6">
@@ -14259,8 +14440,8 @@
         <v>0.8</v>
       </c>
       <c r="Z89" s="6">
-        <f t="shared" si="5"/>
-        <v>159.42561869150151</v>
+        <f>W89</f>
+        <v>142.22395103970482</v>
       </c>
       <c r="AA89" s="6">
         <v>77.87072359385968</v>
@@ -14325,8 +14506,11 @@
       <c r="AU89">
         <v>0.5</v>
       </c>
+      <c r="AW89" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="90" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>246</v>
       </c>
@@ -14394,7 +14578,6 @@
         <v>197.7670255349949</v>
       </c>
       <c r="W90" s="6">
-        <f t="shared" si="6"/>
         <v>155.80250230086676</v>
       </c>
       <c r="X90" s="6">
@@ -14405,8 +14588,8 @@
         <v>0.8</v>
       </c>
       <c r="Z90" s="6">
-        <f t="shared" si="5"/>
-        <v>175.73877431574846</v>
+        <f>W90</f>
+        <v>155.80250230086676</v>
       </c>
       <c r="AA90" s="6">
         <v>41.21189001129185</v>
@@ -14471,8 +14654,11 @@
       <c r="AU90">
         <v>0.5</v>
       </c>
+      <c r="AW90" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="91" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>247</v>
       </c>
@@ -14540,7 +14726,6 @@
         <v>116.91003616433591</v>
       </c>
       <c r="W91" s="6">
-        <f t="shared" si="6"/>
         <v>161.27272639678267</v>
       </c>
       <c r="X91" s="6">
@@ -14551,8 +14736,8 @@
         <v>0.8</v>
       </c>
       <c r="Z91" s="6">
-        <f t="shared" si="5"/>
-        <v>187.03677864585129</v>
+        <f>W91</f>
+        <v>161.27272639678267</v>
       </c>
       <c r="AA91" s="6">
         <v>11.862849818414871</v>
@@ -14617,8 +14802,11 @@
       <c r="AU91">
         <v>0.5</v>
       </c>
+      <c r="AW91" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="92" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>249</v>
       </c>
@@ -14686,7 +14874,6 @@
         <v>155.9588046497083</v>
       </c>
       <c r="W92" s="6">
-        <f t="shared" si="6"/>
         <v>146.67445820250575</v>
       </c>
       <c r="X92" s="6">
@@ -14697,8 +14884,8 @@
         <v>0.8</v>
       </c>
       <c r="Z92" s="6">
-        <f t="shared" si="5"/>
-        <v>166.20710036565779</v>
+        <f>W92</f>
+        <v>146.67445820250575</v>
       </c>
       <c r="AA92" s="6">
         <v>17.844477675710319</v>
@@ -14763,8 +14950,11 @@
       <c r="AU92">
         <v>0.5</v>
       </c>
+      <c r="AW92" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="93" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>26000019</v>
       </c>
@@ -14832,8 +15022,7 @@
         <v>90</v>
       </c>
       <c r="W93" s="6">
-        <f t="shared" si="6"/>
-        <v>68.833333333333329</v>
+        <v>68.83333333333333</v>
       </c>
       <c r="X93" s="6">
         <f t="shared" si="7"/>
@@ -14843,8 +15032,8 @@
         <v>0.8</v>
       </c>
       <c r="Z93" s="6">
-        <f t="shared" si="5"/>
-        <v>84.376248035530793</v>
+        <f>W93</f>
+        <v>68.83333333333333</v>
       </c>
       <c r="AA93" s="6">
         <v>54.085818048646502</v>
@@ -14909,8 +15098,11 @@
       <c r="AU93">
         <v>0.5</v>
       </c>
+      <c r="AW93" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="94" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>34076279</v>
       </c>
@@ -14978,7 +15170,6 @@
         <v>96.180787446792237</v>
       </c>
       <c r="W94" s="6">
-        <f t="shared" si="6"/>
         <v>121.88217264465493</v>
       </c>
       <c r="X94" s="6">
@@ -14989,8 +15180,8 @@
         <v>0.8</v>
       </c>
       <c r="Z94" s="6">
-        <f t="shared" si="5"/>
-        <v>151.90466067695272</v>
+        <f>W94</f>
+        <v>121.88217264465493</v>
       </c>
       <c r="AA94" s="6">
         <v>84.587237159337135</v>
@@ -15055,8 +15246,11 @@
       <c r="AU94">
         <v>0.5</v>
       </c>
+      <c r="AW94" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="95" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>253</v>
       </c>
@@ -15124,7 +15318,6 @@
         <v>137.0218971409486</v>
       </c>
       <c r="W95" s="6">
-        <f t="shared" si="6"/>
         <v>153.06270919736562</v>
       </c>
       <c r="X95" s="6">
@@ -15135,8 +15328,8 @@
         <v>0.8</v>
       </c>
       <c r="Z95" s="6">
-        <f t="shared" si="5"/>
-        <v>176.41262343185269</v>
+        <f>W95</f>
+        <v>153.06270919736562</v>
       </c>
       <c r="AA95" s="6">
         <v>36.846522415845207</v>
@@ -15201,8 +15394,11 @@
       <c r="AU95">
         <v>0.5</v>
       </c>
+      <c r="AW95" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="96" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>255</v>
       </c>
@@ -15270,7 +15466,6 @@
         <v>171.83629703722539</v>
       </c>
       <c r="W96" s="6">
-        <f t="shared" si="6"/>
         <v>153.66402446161374</v>
       </c>
       <c r="X96" s="6">
@@ -15281,8 +15476,8 @@
         <v>0.8</v>
       </c>
       <c r="Z96" s="6">
-        <f t="shared" si="5"/>
-        <v>182.23936130516955</v>
+        <f>W96</f>
+        <v>153.66402446161374</v>
       </c>
       <c r="AA96" s="6">
         <v>70.629291665395058</v>
@@ -15347,8 +15542,11 @@
       <c r="AU96">
         <v>0.5</v>
       </c>
+      <c r="AW96" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="97" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>257</v>
       </c>
@@ -15416,7 +15614,6 @@
         <v>160.404835393274</v>
       </c>
       <c r="W97" s="6">
-        <f t="shared" si="6"/>
         <v>161.61355669410116</v>
       </c>
       <c r="X97" s="6">
@@ -15427,8 +15624,8 @@
         <v>0.8</v>
       </c>
       <c r="Z97" s="6">
-        <f t="shared" si="5"/>
-        <v>181.76953368768778</v>
+        <f>W97</f>
+        <v>161.61355669410116</v>
       </c>
       <c r="AA97" s="6">
         <v>83.950010681478318</v>
@@ -15493,8 +15690,11 @@
       <c r="AU97">
         <v>0.5</v>
       </c>
+      <c r="AW97" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="98" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>26111121</v>
       </c>
@@ -15562,7 +15762,6 @@
         <v>132.65935801100571</v>
       </c>
       <c r="W98" s="6">
-        <f t="shared" si="6"/>
         <v>158.95974778813977</v>
       </c>
       <c r="X98" s="6">
@@ -15573,8 +15772,8 @@
         <v>0.8</v>
       </c>
       <c r="Z98" s="6">
-        <f t="shared" si="5"/>
-        <v>173.8062562608402</v>
+        <f>W98</f>
+        <v>158.95974778813977</v>
       </c>
       <c r="AA98" s="6">
         <v>22.673726615192109</v>
@@ -15639,8 +15838,11 @@
       <c r="AU98">
         <v>0.5</v>
       </c>
+      <c r="AW98" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="99" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>28260092</v>
       </c>
@@ -15708,7 +15910,6 @@
         <v>167.8421032615006</v>
       </c>
       <c r="W99" s="6">
-        <f t="shared" si="6"/>
         <v>157.89597436323675</v>
       </c>
       <c r="X99" s="6">
@@ -15719,8 +15920,8 @@
         <v>0.8</v>
       </c>
       <c r="Z99" s="6">
-        <f t="shared" si="5"/>
-        <v>181.64801538622604</v>
+        <f>W99</f>
+        <v>157.89597436323675</v>
       </c>
       <c r="AA99" s="6">
         <v>64.510940885647145</v>
@@ -15785,8 +15986,11 @@
       <c r="AU99">
         <v>0.5</v>
       </c>
+      <c r="AW99" s="7">
+        <v>0.5</v>
+      </c>
     </row>
-    <row r="100" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>27002211</v>
       </c>
@@ -15854,7 +16058,7 @@
         <v>66</v>
       </c>
       <c r="W100" s="6">
-        <f t="shared" si="6"/>
+        <f>AVERAGE(K100:V100)</f>
         <v>88.666666666666671</v>
       </c>
       <c r="X100" s="6">
@@ -15865,7 +16069,7 @@
         <v>0.8</v>
       </c>
       <c r="Z100" s="6">
-        <f t="shared" si="5"/>
+        <f>NORMINV(Y100,W100,X100)</f>
         <v>150.12475269232195</v>
       </c>
       <c r="AA100" s="6">
@@ -15929,6 +16133,9 @@
         <v>0.4</v>
       </c>
       <c r="AU100">
+        <v>0.5</v>
+      </c>
+      <c r="AW100" s="7">
         <v>0.5</v>
       </c>
     </row>

</xml_diff>